<commit_message>
feat: Introduce multi-source NBA odds scraping and player props ML prediction.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-19.xlsx
+++ b/results/nba_predictions_2025-12-19.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>65.22</v>
+        <v>55.13</v>
       </c>
       <c r="E2" t="n">
-        <v>34.78</v>
+        <v>44.87</v>
       </c>
       <c r="F2" t="n">
-        <v>58.84</v>
+        <v>58.98</v>
       </c>
       <c r="G2" t="n">
-        <v>41.16</v>
+        <v>41.02</v>
       </c>
       <c r="H2" t="n">
         <v>0.32</v>
@@ -593,7 +593,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -607,16 +607,16 @@
       <c r="Q2" t="n">
         <v>0</v>
       </c>
-      <c r="R2" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="S2" t="n">
-        <v>34.8</v>
-      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Tyler Herro (OUT)</t>
+        </is>
+      </c>
       <c r="V2" t="n">
-        <v>9.1</v>
+        <v>3.1</v>
       </c>
       <c r="W2" t="n">
         <v>234.3</v>
@@ -639,16 +639,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>73.33</v>
+        <v>54.12</v>
       </c>
       <c r="E3" t="n">
-        <v>26.67</v>
+        <v>45.88</v>
       </c>
       <c r="F3" t="n">
-        <v>56.86</v>
+        <v>56.8</v>
       </c>
       <c r="G3" t="n">
-        <v>43.14</v>
+        <v>43.2</v>
       </c>
       <c r="H3" t="n">
         <v>-0.1</v>
@@ -670,7 +670,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -684,20 +684,20 @@
       <c r="Q3" t="n">
         <v>0</v>
       </c>
-      <c r="R3" t="n">
-        <v>73.3</v>
-      </c>
-      <c r="S3" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Pacome Dadiet (QUESTIONABLE)</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Johni Broome (DOUBTFUL)</t>
+          <t>Johni Broome (OUT)</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>14</v>
+        <v>2.5</v>
       </c>
       <c r="W3" t="n">
         <v>233.6</v>
@@ -720,16 +720,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>55</v>
+        <v>53.3</v>
       </c>
       <c r="E4" t="n">
-        <v>45</v>
+        <v>46.7</v>
       </c>
       <c r="F4" t="n">
-        <v>55.89</v>
+        <v>56.04</v>
       </c>
       <c r="G4" t="n">
-        <v>44.11</v>
+        <v>43.96</v>
       </c>
       <c r="H4" t="n">
         <v>-0.19</v>
@@ -751,7 +751,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -765,16 +765,16 @@
       <c r="Q4" t="n">
         <v>0</v>
       </c>
-      <c r="R4" t="n">
-        <v>55</v>
-      </c>
-      <c r="S4" t="n">
-        <v>45</v>
-      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Harrison Ingram (OUT)</t>
+        </is>
+      </c>
       <c r="V4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W4" t="n">
         <v>233.8</v>
@@ -797,16 +797,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>65.22</v>
+        <v>54.95</v>
       </c>
       <c r="E5" t="n">
-        <v>34.78</v>
+        <v>45.05</v>
       </c>
       <c r="F5" t="n">
-        <v>58.21</v>
+        <v>58.14</v>
       </c>
       <c r="G5" t="n">
-        <v>41.79</v>
+        <v>41.86</v>
       </c>
       <c r="H5" t="n">
         <v>0.09</v>
@@ -828,7 +828,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -842,12 +842,8 @@
       <c r="Q5" t="n">
         <v>0</v>
       </c>
-      <c r="R5" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="S5" t="n">
-        <v>34.8</v>
-      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>Chris Livingston (OUT)</t>
@@ -859,7 +855,7 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>9.1</v>
+        <v>3</v>
       </c>
       <c r="W5" t="n">
         <v>233.8</v>
@@ -882,16 +878,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>32.43</v>
+        <v>52.3</v>
       </c>
       <c r="E6" t="n">
-        <v>67.56999999999999</v>
+        <v>47.7</v>
       </c>
       <c r="F6" t="n">
-        <v>54.98</v>
+        <v>54.91</v>
       </c>
       <c r="G6" t="n">
-        <v>45.02</v>
+        <v>45.09</v>
       </c>
       <c r="H6" t="n">
         <v>-0.04</v>
@@ -913,7 +909,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -927,20 +923,20 @@
       <c r="Q6" t="n">
         <v>0</v>
       </c>
-      <c r="R6" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="S6" t="n">
-        <v>67.59999999999999</v>
-      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>Joan Beringer (OUT)</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Thomas Sorber (OUT)</t>
+        </is>
+      </c>
       <c r="V6" t="n">
-        <v>-10.5</v>
+        <v>1.4</v>
       </c>
       <c r="W6" t="n">
         <v>234.5</v>

</xml_diff>